<commit_message>
updated selenium test results excel file in test-results folder
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="195">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -502,6 +502,147 @@
   </si>
   <si>
     <t>2026-10-05T15:07:32.246002500</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:01:56.472591100</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:07.326166800</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:09.712842700</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:10.544744</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:18.310268500</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:22.301361900</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:24.878665600</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:27.591749100</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:31.951677800</t>
+  </si>
+  <si>
+    <t>TC-PROD-004</t>
+  </si>
+  <si>
+    <t>Remove an added product from the shopping cart</t>
+  </si>
+  <si>
+    <t>Authenticated user should be able to remove a product from the cart.</t>
+  </si>
+  <si>
+    <t>Product 'Campus 00' was removed successfully from the Shopping Cart.</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:36.987768400</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:38.279116700</t>
+  </si>
+  <si>
+    <t>2026-10-06T23:02:42.018673200</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:06.475526700</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:16.097560900</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:18.953777100</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:20.320187800</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:27.932114700</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:31.778498200</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:33.809659700</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:35.710932300</t>
+  </si>
+  <si>
+    <t>TC-PROD-006</t>
+  </si>
+  <si>
+    <t>Verify product information is displayed</t>
+  </si>
+  <si>
+    <t>Product card should display product name and essential information.</t>
+  </si>
+  <si>
+    <t>Product information was displayed successfully.</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:41.970722800</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:45.295959200</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:49.718165400</t>
+  </si>
+  <si>
+    <t>Product price is missing. expected [true] but found [false]</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:46:50.677455300</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:55:47.236690300</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:55:58.467525500</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:01.490278500</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:02.595181400</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:10.575471700</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:14.101485100</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:16.249502900</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:18.409547</t>
+  </si>
+  <si>
+    <t>TC-PROD-005</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:25.262155100</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:27.662160300</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:34.133819900</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:35.157953200</t>
+  </si>
+  <si>
+    <t>2026-10-07T11:56:39.042194</t>
   </si>
 </sst>
 </file>
@@ -546,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F113"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2069,6 +2210,746 @@
         <v>147</v>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B77" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C77" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D77" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E77" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F77" t="s" s="0">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C78" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D78" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E78" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F78" t="s" s="0">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C79" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D79" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E79" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F79" t="s" s="0">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C80" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D80" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E80" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F80" t="s" s="0">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C81" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D81" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E81" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F81" t="s" s="0">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C82" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D82" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E82" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F82" t="s" s="0">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C83" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D83" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E83" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F83" t="s" s="0">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C84" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D84" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E84" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F84" t="s" s="0">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C85" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D85" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E85" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F85" t="s" s="0">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C86" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D86" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E86" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F86" t="s" s="0">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C87" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D87" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E87" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F87" t="s" s="0">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C88" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D88" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E88" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F88" t="s" s="0">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C89" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D89" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E89" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F89" t="s" s="0">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C90" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E90" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F90" t="s" s="0">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C91" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D91" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E91" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F91" t="s" s="0">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C92" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D92" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E92" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F92" t="s" s="0">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C93" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D93" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E93" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F93" t="s" s="0">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C94" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D94" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E94" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F94" t="s" s="0">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C95" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D95" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E95" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s" s="0">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C96" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D96" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E96" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F96" t="s" s="0">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s" s="0">
+        <v>172</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C97" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D97" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E97" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F97" t="s" s="0">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C98" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D98" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E98" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F98" t="s" s="0">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C99" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D99" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E99" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F99" t="s" s="0">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C100" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D100" t="s" s="0">
+        <v>179</v>
+      </c>
+      <c r="E100" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F100" t="s" s="0">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C101" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D101" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E101" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F101" t="s" s="0">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C102" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D102" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E102" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F102" t="s" s="0">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C103" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D103" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E103" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F103" t="s" s="0">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B104" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C104" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D104" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E104" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F104" t="s" s="0">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B105" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C105" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D105" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E105" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F105" t="s" s="0">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C106" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D106" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E106" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F106" t="s" s="0">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C107" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D107" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E107" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F107" t="s" s="0">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C108" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D108" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E108" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F108" t="s" s="0">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B109" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C109" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D109" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E109" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F109" t="s" s="0">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C110" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D110" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E110" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F110" t="s" s="0">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C111" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D111" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E111" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F111" t="s" s="0">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C112" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D112" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E112" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F112" t="s" s="0">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C113" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D113" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E113" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F113" t="s" s="0">
+        <v>194</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added test casses TC-LOGIN-004 and TC-LOGIN-005 in file LoginTest.java
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="218">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -643,6 +643,75 @@
   </si>
   <si>
     <t>2026-10-07T11:56:39.042194</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:23.534594</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:25.460765</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:26.211183</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:28.400834</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:28.783106</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:30.430544</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-005</t>
+  </si>
+  <si>
+    <t>Login with invalid credentials</t>
+  </si>
+  <si>
+    <t>Invalid credentials should not create an authenticated session.</t>
+  </si>
+  <si>
+    <t>Invalid credentials did not authenticate the user.</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:33.834539</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-004</t>
+  </si>
+  <si>
+    <t>Verify login page elements</t>
+  </si>
+  <si>
+    <t>Email, password, remember-me and Sign in controls are displayed.</t>
+  </si>
+  <si>
+    <t>All login page controls are displayed.</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:33.944233</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:34.637093</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:34.984546</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:35.035361</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:37.013619</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:38.151397</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:38.719223</t>
+  </si>
+  <si>
+    <t>2026-10-08T20:22:39.199333</t>
   </si>
 </sst>
 </file>
@@ -687,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2950,6 +3019,306 @@
         <v>194</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C114" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D114" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E114" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F114" t="s" s="0">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C115" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D115" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E115" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F115" t="s" s="0">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C116" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F116" t="s" s="0">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C117" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F117" t="s" s="0">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B118" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C118" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D118" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E118" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F118" t="s" s="0">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B119" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C119" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D119" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E119" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F119" t="s" s="0">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C120" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D120" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E120" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F120" t="s" s="0">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C121" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D121" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E121" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F121" t="s" s="0">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B122" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C122" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D122" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E122" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F122" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B123" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C123" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D123" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E123" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F123" t="s" s="0">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B124" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C124" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D124" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E124" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F124" t="s" s="0">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B125" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C125" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D125" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E125" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F125" t="s" s="0">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B126" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C126" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D126" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E126" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F126" t="s" s="0">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B127" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C127" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D127" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E127" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F127" t="s" s="0">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B128" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C128" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D128" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E128" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F128" t="s" s="0">
+        <v>217</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Add tests/CartTest.java to test cart updates, totals, removal, and persistence
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="243">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -712,6 +712,88 @@
   </si>
   <si>
     <t>2026-10-08T20:22:39.199333</t>
+  </si>
+  <si>
+    <t>TC-CART-004</t>
+  </si>
+  <si>
+    <t>Cart contents persist after page reload</t>
+  </si>
+  <si>
+    <t>The same cart item and quantity remain after reload.</t>
+  </si>
+  <si>
+    <t>unknown error: net::ERR_CONNECTION_REFUSED
+  (Session info: chrome=154.0.8037.98)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.12.1'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [63e4c304747bde681d143e4b6b6f6f84, get {url=http://localhost:5173}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 154.0.8037.98, chrome: {chromedriverVersion: 154.0.8037.92 (334b65d254cc..., userDataDir: C:\Users\ASHISH~1\AppData\L...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:62610}, goog:processID: 20808, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:62610/devtoo..., se:cdpVersion: 154.0.8037.98, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 63e4c304747bde681d143e4b6b6f6f84</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:37:54.545257300</t>
+  </si>
+  <si>
+    <t>TC-CART-001</t>
+  </si>
+  <si>
+    <t>Increase and decrease cart item quantity</t>
+  </si>
+  <si>
+    <t>Quantity increments and decrements correctly for a cart item.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:37:54.858021200</t>
+  </si>
+  <si>
+    <t>TC-CART-003</t>
+  </si>
+  <si>
+    <t>Remove an item from the shopping cart</t>
+  </si>
+  <si>
+    <t>Removed item no longer appears in the cart.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:37:55.040151100</t>
+  </si>
+  <si>
+    <t>TC-CART-002</t>
+  </si>
+  <si>
+    <t>Verify cart subtotal, shipping and total</t>
+  </si>
+  <si>
+    <t>Subtotal equals item price times quantity and total equals subtotal plus ₹150 shipping.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:37:55.242561500</t>
+  </si>
+  <si>
+    <t>Product 'Campus 00' remained in cart with quantity 2 after reload.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:39:16.100220600</t>
+  </si>
+  <si>
+    <t>Quantity increased to 4 and returned to 3.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:39:21.037511800</t>
+  </si>
+  <si>
+    <t>Removed product 'Campus 00' is no longer displayed.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:39:25.135569200</t>
+  </si>
+  <si>
+    <t>Subtotal ₹6500.00 + shipping ₹150.00 = total ₹6650.00.</t>
+  </si>
+  <si>
+    <t>2026-10-09T17:39:28.120071100</t>
   </si>
 </sst>
 </file>
@@ -756,7 +838,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F136"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3319,6 +3401,166 @@
         <v>217</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B129" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C129" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D129" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="E129" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F129" t="s" s="0">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B130" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C130" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D130" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="E130" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F130" t="s" s="0">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B131" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C131" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D131" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="E131" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F131" t="s" s="0">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B132" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C132" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D132" t="s" s="0">
+        <v>221</v>
+      </c>
+      <c r="E132" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F132" t="s" s="0">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B133" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C133" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D133" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E133" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F133" t="s" s="0">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B134" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C134" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D134" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E134" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F134" t="s" s="0">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B135" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C135" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D135" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E135" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F135" t="s" s="0">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B136" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C136" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D136" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E136" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F136" t="s" s="0">
+        <v>242</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added TC-HOME-003 to HomeTest.java and updated excel sheet
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="287">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -794,6 +794,138 @@
   </si>
   <si>
     <t>2026-10-09T17:39:28.120071100</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:25.615425</t>
+  </si>
+  <si>
+    <t>TC-HOME-002</t>
+  </si>
+  <si>
+    <t>Verify home page content</t>
+  </si>
+  <si>
+    <t>Home page displays main heading, description and Shop Now button.</t>
+  </si>
+  <si>
+    <t>Home page content is displayed correctly.</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:25.782012</t>
+  </si>
+  <si>
+    <t>TC-HOME-003</t>
+  </si>
+  <si>
+    <t>Verify Shop Now navigation</t>
+  </si>
+  <si>
+    <t>Clicking Shop Now navigates user to the Shop page.</t>
+  </si>
+  <si>
+    <t>Shop Now successfully navigated to /shop.</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:27.225374</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:28.735274</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:29.508479</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:31.685857</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:32.073424</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:33.728780</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:36.979654</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:37.093381</t>
+  </si>
+  <si>
+    <t>TC-LOGIN-006</t>
+  </si>
+  <si>
+    <t>Verify Remember Me checkbox</t>
+  </si>
+  <si>
+    <t>Remember Me checkbox can be selected and deselected.</t>
+  </si>
+  <si>
+    <t>Remember Me checkbox works correctly.</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:37.175905</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:37.871064</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:38.210068</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:38.266201</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:40.173103</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:41.321053</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:41.874371</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:42.337292</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:47.185433</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:50.715951</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:53.707839</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:22:56.133954</t>
+  </si>
+  <si>
+    <t>TC-SELL-001</t>
+  </si>
+  <si>
+    <t>Validate required fields on Sell form</t>
+  </si>
+  <si>
+    <t>Form cannot be submitted when required fields are empty.</t>
+  </si>
+  <si>
+    <t>Browser form validation rejected submission with required fields empty.</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:23:01.707988</t>
+  </si>
+  <si>
+    <t>TC-SELL-002</t>
+  </si>
+  <si>
+    <t>Create a listing and verify it in My Listings</t>
+  </si>
+  <si>
+    <t>Valid listing is saved and displayed in the authenticated user's My Listings.</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791723182412' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-11T18:23:04.305259</t>
   </si>
 </sst>
 </file>
@@ -838,7 +970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3561,6 +3693,486 @@
         <v>242</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B137" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C137" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D137" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E137" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F137" t="s" s="0">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B138" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C138" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D138" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E138" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F138" t="s" s="0">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B139" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C139" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D139" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E139" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F139" t="s" s="0">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B140" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C140" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D140" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E140" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F140" t="s" s="0">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B141" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C141" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D141" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E141" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F141" t="s" s="0">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B142" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C142" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D142" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E142" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F142" t="s" s="0">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B143" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C143" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D143" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E143" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F143" t="s" s="0">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B144" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C144" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D144" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E144" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s" s="0">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B145" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C145" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D145" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E145" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F145" t="s" s="0">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B146" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C146" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D146" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E146" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F146" t="s" s="0">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B147" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C147" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D147" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E147" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F147" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B148" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C148" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D148" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E148" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F148" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B149" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C149" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D149" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E149" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F149" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B150" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C150" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D150" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E150" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F150" t="s" s="0">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B151" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C151" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D151" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E151" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F151" t="s" s="0">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B152" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C152" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D152" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E152" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F152" t="s" s="0">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B153" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C153" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D153" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E153" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F153" t="s" s="0">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B154" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C154" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D154" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E154" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F154" t="s" s="0">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B155" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C155" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D155" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E155" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F155" t="s" s="0">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B156" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C156" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D156" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E156" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F156" t="s" s="0">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B157" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C157" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D157" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E157" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F157" t="s" s="0">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B158" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C158" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D158" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E158" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F158" t="s" s="0">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B159" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C159" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D159" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E159" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F159" t="s" s="0">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B160" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C160" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D160" t="s" s="0">
+        <v>285</v>
+      </c>
+      <c r="E160" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F160" t="s" s="0">
+        <v>286</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Test case TC-SELL-003 and TC-SELL-004 added to SellTest.java and updated the excel sheet.
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="379">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -926,6 +926,294 @@
   </si>
   <si>
     <t>2026-10-11T18:23:04.305259</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:43.303124</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:43.481496</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:43.931878</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:45.572617</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:46.357998</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:48.562801</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:48.949059</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:50.590242</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:51.567981</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:51.684686</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:51.779997</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:52.162041</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:52.481442</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:52.523227</t>
+  </si>
+  <si>
+    <t>TC-LIST-003</t>
+  </si>
+  <si>
+    <t>Cancel listing deletion</t>
+  </si>
+  <si>
+    <t>Cancelling deletion keeps the listing visible.</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791908574140' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:56.542085</t>
+  </si>
+  <si>
+    <t>TC-LIST-002</t>
+  </si>
+  <si>
+    <t>Delete a listing after confirmation</t>
+  </si>
+  <si>
+    <t>Confirming deletion removes the listing from My Listings.</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791908577789'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:52:59.622150</t>
+  </si>
+  <si>
+    <t>TC-LIST-004</t>
+  </si>
+  <si>
+    <t>Verify listing ownership for authenticated user</t>
+  </si>
+  <si>
+    <t>Created listing seller_id matches the authenticated user's user_id.</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791908580305' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:02.227875</t>
+  </si>
+  <si>
+    <t>TC-LIST-001</t>
+  </si>
+  <si>
+    <t>Update a listing status</t>
+  </si>
+  <si>
+    <t>Changing listing status updates the displayed status.</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h3[normalize-space()='Selenium QA Item 1791908582926'], but... org.openqa.selenium.NoSuchElementException: no such element: Unable to locate element: {"method":"xpath","selector":"//h3[normalize-space()='Selenium QA Item 1791908582926']"}.
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 155.0.8059.39, chrome: {chromedriverVersion: 155.0.8059.39 (3ff7ac5a9224..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:49353}, goog:processID: 3602, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:49353/devtoo..., se:cdpVersion: 155.0.8059.39, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 3dae5b0e9dc7aec7c68c86a378460d25</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:14.980773</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:18.825246</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:20.066504</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:20.372557</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:20.617610</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:24.471442</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:27.999525</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:30.974264</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:33.412459</t>
+  </si>
+  <si>
+    <t>TC-SELL-004</t>
+  </si>
+  <si>
+    <t>Verify listing dropdowns</t>
+  </si>
+  <si>
+    <t>Dropdowns have the correct defaults and options.</t>
+  </si>
+  <si>
+    <t>Dropdown defaults and options are correct.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:35.570738</t>
+  </si>
+  <si>
+    <t>TC-SELL-003</t>
+  </si>
+  <si>
+    <t>Reject negative selling price</t>
+  </si>
+  <si>
+    <t>Negative selling price fails browser validation.</t>
+  </si>
+  <si>
+    <t>Browser validation rejected the negative price.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:36.863526</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:38.173312</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791908618868' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:53:40.750270</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:19.656183</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:19.828748</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:20.464114</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:22.057796</t>
+  </si>
+  <si>
+    <t>Inventory loaded with 14 product card(s).</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:22.854461</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:25.047652</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:25.435578</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:27.072430</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:29.106400</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:29.214179</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:29.331746</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:29.712074</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:30.056904</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:30.113346</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791908671742' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:33.121465</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791908674359'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:36.192600</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791908676893' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:38.829836</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h3[normalize-space()='Selenium QA Item 1791908679534'], but... org.openqa.selenium.NoSuchElementException: no such element: Unable to locate element: {"method":"xpath","selector":"//h3[normalize-space()='Selenium QA Item 1791908679534']"}.
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 155.0.8059.39, chrome: {chromedriverVersion: 155.0.8059.39 (3ff7ac5a9224..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:49609}, goog:processID: 4179, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:49609/devtoo..., se:cdpVersion: 155.0.8059.39, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 9ecf7c8836c2de09dead780022e00c9c</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:51.562512</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:56.931847</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:58.085163</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:58.349929</t>
+  </si>
+  <si>
+    <t>Protected route did not redirect to /login. expected [true] but found [false]</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:54:58.500930</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:02.391422</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:05.884048</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:08.855688</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:11.302975</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:13.503477</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:14.779166</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:16.081692</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791908716786' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T21:55:18.656380</t>
   </si>
 </sst>
 </file>
@@ -970,7 +1258,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F160"/>
+  <dimension ref="A1:F220"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -4173,6 +4461,1206 @@
         <v>286</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B161" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C161" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D161" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E161" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F161" t="s" s="0">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B162" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C162" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D162" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E162" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F162" t="s" s="0">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B163" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C163" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D163" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E163" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F163" t="s" s="0">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B164" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C164" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D164" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E164" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F164" t="s" s="0">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B165" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C165" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D165" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E165" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F165" t="s" s="0">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B166" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C166" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D166" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E166" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F166" t="s" s="0">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B167" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C167" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D167" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E167" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F167" t="s" s="0">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B168" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C168" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D168" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E168" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F168" t="s" s="0">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B169" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C169" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D169" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E169" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F169" t="s" s="0">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B170" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C170" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D170" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E170" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F170" t="s" s="0">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B171" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C171" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D171" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E171" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F171" t="s" s="0">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B172" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C172" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D172" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E172" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F172" t="s" s="0">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B173" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C173" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D173" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E173" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F173" t="s" s="0">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B174" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C174" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D174" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E174" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F174" t="s" s="0">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B175" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C175" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D175" t="s" s="0">
+        <v>304</v>
+      </c>
+      <c r="E175" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F175" t="s" s="0">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B176" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C176" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D176" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="E176" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F176" t="s" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B177" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C177" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D177" t="s" s="0">
+        <v>314</v>
+      </c>
+      <c r="E177" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F177" t="s" s="0">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B178" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C178" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D178" t="s" s="0">
+        <v>319</v>
+      </c>
+      <c r="E178" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F178" t="s" s="0">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B179" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C179" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D179" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E179" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F179" t="s" s="0">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B180" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C180" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D180" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E180" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F180" t="s" s="0">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B181" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C181" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D181" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E181" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F181" t="s" s="0">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B182" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C182" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D182" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E182" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F182" t="s" s="0">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B183" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C183" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D183" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E183" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F183" t="s" s="0">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B184" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C184" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D184" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E184" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F184" t="s" s="0">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B185" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C185" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D185" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E185" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F185" t="s" s="0">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B186" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C186" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D186" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E186" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F186" t="s" s="0">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B187" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C187" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D187" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E187" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F187" t="s" s="0">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B188" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C188" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D188" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E188" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F188" t="s" s="0">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B189" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C189" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D189" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E189" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F189" t="s" s="0">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B190" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C190" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D190" t="s" s="0">
+        <v>340</v>
+      </c>
+      <c r="E190" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F190" t="s" s="0">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B191" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C191" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D191" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E191" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F191" t="s" s="0">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B192" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C192" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D192" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E192" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F192" t="s" s="0">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B193" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C193" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D193" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E193" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F193" t="s" s="0">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B194" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C194" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D194" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E194" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F194" t="s" s="0">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B195" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C195" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D195" t="s" s="0">
+        <v>346</v>
+      </c>
+      <c r="E195" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F195" t="s" s="0">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B196" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C196" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D196" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E196" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F196" t="s" s="0">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B197" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C197" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D197" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E197" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F197" t="s" s="0">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B198" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C198" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D198" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E198" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F198" t="s" s="0">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B199" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C199" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D199" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E199" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F199" t="s" s="0">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B200" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C200" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D200" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E200" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F200" t="s" s="0">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B201" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C201" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D201" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E201" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F201" t="s" s="0">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B202" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C202" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D202" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E202" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F202" t="s" s="0">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B203" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C203" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D203" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E203" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F203" t="s" s="0">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B204" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C204" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D204" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E204" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F204" t="s" s="0">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B205" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C205" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D205" t="s" s="0">
+        <v>357</v>
+      </c>
+      <c r="E205" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F205" t="s" s="0">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B206" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C206" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D206" t="s" s="0">
+        <v>359</v>
+      </c>
+      <c r="E206" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F206" t="s" s="0">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B207" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C207" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D207" t="s" s="0">
+        <v>361</v>
+      </c>
+      <c r="E207" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F207" t="s" s="0">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B208" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C208" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D208" t="s" s="0">
+        <v>363</v>
+      </c>
+      <c r="E208" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F208" t="s" s="0">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B209" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C209" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D209" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E209" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F209" t="s" s="0">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B210" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C210" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D210" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="E210" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F210" t="s" s="0">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B211" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C211" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D211" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E211" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F211" t="s" s="0">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B212" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C212" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D212" t="s" s="0">
+        <v>368</v>
+      </c>
+      <c r="E212" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F212" t="s" s="0">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B213" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C213" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D213" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E213" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F213" t="s" s="0">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B214" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C214" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D214" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E214" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F214" t="s" s="0">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B215" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C215" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D215" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E215" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F215" t="s" s="0">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B216" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C216" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D216" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E216" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F216" t="s" s="0">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B217" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C217" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D217" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E217" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F217" t="s" s="0">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B218" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C218" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D218" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E218" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F218" t="s" s="0">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B219" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C219" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D219" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E219" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F219" t="s" s="0">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B220" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C220" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D220" t="s" s="0">
+        <v>377</v>
+      </c>
+      <c r="E220" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F220" t="s" s="0">
+        <v>378</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Solving Listeing and navigation test case error
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="525">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -1214,6 +1214,444 @@
   </si>
   <si>
     <t>2026-10-13T21:55:18.656380</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:07.577702</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:07.766735</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:08.737581</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:10.676534</t>
+  </si>
+  <si>
+    <t>Inventory loaded with 16 product card(s).</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:11.504615</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:13.713245</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:14.109567</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:15.741536</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:17.762580</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:17.863400</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:17.982146</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:18.401786</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:18.742315</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:18.799693</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791909200386' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:21.758877</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791909203002'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:24.837973</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791909205538' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:27.456239</t>
+  </si>
+  <si>
+    <t>Status update failed in the application. Check the backend terminal for the PUT request error.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:30.001286</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:32.611147</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:43.608585</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:44.442136</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:44.681724</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:49.390787</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:52.931291</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:55.888679</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:03:58.357139</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:04:00.385818</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:04:01.655216</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:04:02.950257</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791909243631' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:04:05.489946</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:20.399023</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:20.593496</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:22.089114</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:24.307193</t>
+  </si>
+  <si>
+    <t>Inventory loaded with 18 product card(s).</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:25.348292</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:27.579817</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:27.982319</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:29.631613</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:31.684302</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:31.800886</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:31.893002</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:32.273117</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:32.623128</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:32.683445</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791910114363' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:35.719184</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791910116978'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:38.824809</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791910119535' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:41.463898</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:44.006675</t>
+  </si>
+  <si>
+    <t>Navigate using Shop Now</t>
+  </si>
+  <si>
+    <t>Shop Now should open /shop.</t>
+  </si>
+  <si>
+    <t>Shop Now successfully opened /shop.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:45.512122</t>
+  </si>
+  <si>
+    <t>Authenticated user should reach /shop.</t>
+  </si>
+  <si>
+    <t>Successfully navigated to /shop.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:46.311535</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:47.271889</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:48.014358</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:51.928273</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:55.449900</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:18:58.395783</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:19:00.883653</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:19:03.089124</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:19:04.347743</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:19:05.621577</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791910146313' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:19:08.193855</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:10.453491</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:10.630603</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:13.719015</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:15.456146</t>
+  </si>
+  <si>
+    <t>Inventory loaded with 20 product card(s).</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:16.263453</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:18.471468</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:18.881269</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:20.529469</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:21.351182</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:21.465308</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:21.562362</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:21.955977</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:22.307619</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:22.361065</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791910224736' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:26.113162</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791910227355'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:29.186811</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791910229870' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:31.792148</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:34.322822</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:36.537555</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:37.383589</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:38.360908</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:39.102048</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:43.400555</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:46.912619</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:49.882558</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:52.328950</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:54.329897</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:55.577486</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:56.872433</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791910257568' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:20:59.426086</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:46.623616</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:46.795857</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:49.871824</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:52.648755</t>
+  </si>
+  <si>
+    <t>Inventory loaded with 22 product card(s).</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:53.416839</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:55.621833</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:56.019085</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:57.666789</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:58.495840</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:58.596641</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:58.744677</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:59.151144</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:59.493001</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:27:59.548241</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1791910680944' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:02.305476</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1791910683564'.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:05.410620</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1791910686120' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:08.051975</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:10.574774</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:11.872931</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:12.675865</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:13.671820</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:14.417448</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:22.238185</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:25.776895</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:28.755141</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:31.188345</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:33.253814</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:34.537408</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:36.351608</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1791910717046' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-13T22:28:38.925480</t>
   </si>
 </sst>
 </file>
@@ -1258,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F220"/>
+  <dimension ref="A1:F340"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -5661,6 +6099,2406 @@
         <v>378</v>
       </c>
     </row>
+    <row r="221">
+      <c r="A221" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B221" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C221" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D221" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E221" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F221" t="s" s="0">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B222" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C222" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D222" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E222" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F222" t="s" s="0">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B223" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C223" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D223" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E223" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F223" t="s" s="0">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B224" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C224" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D224" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E224" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F224" t="s" s="0">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B225" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C225" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D225" t="s" s="0">
+        <v>383</v>
+      </c>
+      <c r="E225" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F225" t="s" s="0">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B226" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C226" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D226" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E226" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F226" t="s" s="0">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B227" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C227" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D227" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E227" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F227" t="s" s="0">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B228" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C228" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D228" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E228" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F228" t="s" s="0">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B229" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C229" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D229" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E229" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F229" t="s" s="0">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B230" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C230" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D230" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E230" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F230" t="s" s="0">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B231" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C231" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D231" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E231" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F231" t="s" s="0">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B232" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C232" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D232" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E232" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F232" t="s" s="0">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B233" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C233" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D233" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E233" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F233" t="s" s="0">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B234" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C234" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D234" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E234" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F234" t="s" s="0">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B235" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C235" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D235" t="s" s="0">
+        <v>394</v>
+      </c>
+      <c r="E235" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F235" t="s" s="0">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B236" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C236" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D236" t="s" s="0">
+        <v>396</v>
+      </c>
+      <c r="E236" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F236" t="s" s="0">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B237" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C237" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D237" t="s" s="0">
+        <v>398</v>
+      </c>
+      <c r="E237" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F237" t="s" s="0">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B238" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C238" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D238" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="E238" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F238" t="s" s="0">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B239" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C239" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="D239" t="s" s="0">
+        <v>99</v>
+      </c>
+      <c r="E239" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F239" t="s" s="0">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B240" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="C240" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="D240" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E240" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F240" t="s" s="0">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B241" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C241" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D241" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E241" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F241" t="s" s="0">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B242" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C242" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D242" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E242" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F242" t="s" s="0">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B243" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C243" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D243" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E243" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F243" t="s" s="0">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B244" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C244" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D244" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E244" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F244" t="s" s="0">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B245" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C245" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D245" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E245" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F245" t="s" s="0">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B246" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C246" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D246" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E246" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F246" t="s" s="0">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B247" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C247" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D247" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E247" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F247" t="s" s="0">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B248" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C248" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D248" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E248" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F248" t="s" s="0">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B249" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C249" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D249" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E249" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F249" t="s" s="0">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B250" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C250" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D250" t="s" s="0">
+        <v>413</v>
+      </c>
+      <c r="E250" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F250" t="s" s="0">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B251" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C251" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D251" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E251" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F251" t="s" s="0">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B252" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C252" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D252" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E252" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F252" t="s" s="0">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B253" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C253" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D253" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E253" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F253" t="s" s="0">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B254" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C254" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D254" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E254" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F254" t="s" s="0">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B255" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C255" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D255" t="s" s="0">
+        <v>419</v>
+      </c>
+      <c r="E255" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F255" t="s" s="0">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B256" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C256" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D256" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E256" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F256" t="s" s="0">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B257" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C257" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D257" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E257" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F257" t="s" s="0">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B258" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C258" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D258" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E258" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F258" t="s" s="0">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B259" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C259" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D259" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E259" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F259" t="s" s="0">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B260" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C260" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D260" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E260" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F260" t="s" s="0">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B261" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C261" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D261" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E261" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F261" t="s" s="0">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B262" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C262" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D262" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E262" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F262" t="s" s="0">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B263" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C263" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D263" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E263" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F263" t="s" s="0">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B264" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C264" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D264" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E264" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F264" t="s" s="0">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B265" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C265" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D265" t="s" s="0">
+        <v>430</v>
+      </c>
+      <c r="E265" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F265" t="s" s="0">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B266" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C266" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D266" t="s" s="0">
+        <v>432</v>
+      </c>
+      <c r="E266" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F266" t="s" s="0">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B267" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C267" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D267" t="s" s="0">
+        <v>434</v>
+      </c>
+      <c r="E267" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F267" t="s" s="0">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B268" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C268" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D268" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="E268" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F268" t="s" s="0">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B269" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C269" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D269" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E269" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F269" t="s" s="0">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B270" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C270" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D270" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E270" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F270" t="s" s="0">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B271" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C271" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D271" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E271" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F271" t="s" s="0">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B272" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C272" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D272" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E272" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F272" t="s" s="0">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B273" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C273" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D273" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E273" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F273" t="s" s="0">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B274" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C274" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D274" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E274" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F274" t="s" s="0">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B275" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C275" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D275" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E275" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F275" t="s" s="0">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B276" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C276" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D276" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E276" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F276" t="s" s="0">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B277" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C277" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D277" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E277" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F277" t="s" s="0">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B278" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C278" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D278" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E278" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F278" t="s" s="0">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B279" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C279" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D279" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E279" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F279" t="s" s="0">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B280" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C280" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D280" t="s" s="0">
+        <v>453</v>
+      </c>
+      <c r="E280" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F280" t="s" s="0">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B281" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C281" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D281" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E281" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F281" t="s" s="0">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B282" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C282" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D282" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E282" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F282" t="s" s="0">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B283" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C283" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D283" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E283" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F283" t="s" s="0">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B284" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C284" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D284" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E284" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F284" t="s" s="0">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B285" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C285" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D285" t="s" s="0">
+        <v>459</v>
+      </c>
+      <c r="E285" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F285" t="s" s="0">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B286" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C286" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D286" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E286" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F286" t="s" s="0">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B287" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C287" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D287" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E287" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F287" t="s" s="0">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B288" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C288" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D288" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E288" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F288" t="s" s="0">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B289" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C289" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D289" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E289" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F289" t="s" s="0">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B290" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C290" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D290" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E290" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F290" t="s" s="0">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B291" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C291" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D291" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E291" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F291" t="s" s="0">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B292" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C292" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D292" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E292" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F292" t="s" s="0">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B293" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C293" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D293" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E293" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F293" t="s" s="0">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B294" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C294" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D294" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E294" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F294" t="s" s="0">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B295" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C295" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D295" t="s" s="0">
+        <v>470</v>
+      </c>
+      <c r="E295" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F295" t="s" s="0">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B296" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C296" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D296" t="s" s="0">
+        <v>472</v>
+      </c>
+      <c r="E296" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F296" t="s" s="0">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B297" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C297" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D297" t="s" s="0">
+        <v>474</v>
+      </c>
+      <c r="E297" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F297" t="s" s="0">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B298" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C298" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D298" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="E298" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F298" t="s" s="0">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B299" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C299" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D299" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E299" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F299" t="s" s="0">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B300" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C300" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D300" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E300" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F300" t="s" s="0">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B301" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C301" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D301" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E301" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F301" t="s" s="0">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B302" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C302" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D302" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E302" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F302" t="s" s="0">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B303" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C303" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D303" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E303" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F303" t="s" s="0">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B304" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C304" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D304" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E304" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F304" t="s" s="0">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B305" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C305" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D305" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E305" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F305" t="s" s="0">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B306" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C306" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D306" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E306" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F306" t="s" s="0">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B307" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C307" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D307" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E307" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F307" t="s" s="0">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B308" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C308" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D308" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E308" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F308" t="s" s="0">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B309" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C309" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D309" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E309" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F309" t="s" s="0">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B310" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C310" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D310" t="s" s="0">
+        <v>488</v>
+      </c>
+      <c r="E310" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F310" t="s" s="0">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B311" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C311" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D311" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E311" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F311" t="s" s="0">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B312" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C312" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D312" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E312" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F312" t="s" s="0">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B313" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C313" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D313" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E313" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F313" t="s" s="0">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B314" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C314" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D314" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E314" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F314" t="s" s="0">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B315" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C315" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D315" t="s" s="0">
+        <v>494</v>
+      </c>
+      <c r="E315" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F315" t="s" s="0">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B316" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C316" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D316" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E316" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F316" t="s" s="0">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B317" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C317" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D317" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E317" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F317" t="s" s="0">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B318" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C318" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D318" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E318" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F318" t="s" s="0">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B319" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C319" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D319" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E319" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F319" t="s" s="0">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B320" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C320" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D320" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E320" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F320" t="s" s="0">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B321" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C321" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D321" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E321" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F321" t="s" s="0">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B322" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C322" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D322" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E322" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F322" t="s" s="0">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B323" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C323" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D323" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E323" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F323" t="s" s="0">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B324" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C324" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D324" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E324" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F324" t="s" s="0">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B325" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C325" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D325" t="s" s="0">
+        <v>505</v>
+      </c>
+      <c r="E325" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F325" t="s" s="0">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B326" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C326" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D326" t="s" s="0">
+        <v>507</v>
+      </c>
+      <c r="E326" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F326" t="s" s="0">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B327" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C327" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D327" t="s" s="0">
+        <v>509</v>
+      </c>
+      <c r="E327" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F327" t="s" s="0">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B328" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C328" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D328" t="s" s="0">
+        <v>400</v>
+      </c>
+      <c r="E328" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F328" t="s" s="0">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B329" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C329" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D329" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E329" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F329" t="s" s="0">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B330" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C330" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D330" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E330" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F330" t="s" s="0">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B331" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C331" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D331" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E331" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F331" t="s" s="0">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B332" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C332" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D332" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E332" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F332" t="s" s="0">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B333" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C333" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D333" t="s" s="0">
+        <v>235</v>
+      </c>
+      <c r="E333" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F333" t="s" s="0">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B334" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C334" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D334" t="s" s="0">
+        <v>237</v>
+      </c>
+      <c r="E334" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F334" t="s" s="0">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B335" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C335" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D335" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E335" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F335" t="s" s="0">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B336" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C336" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D336" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E336" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F336" t="s" s="0">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B337" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C337" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D337" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E337" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F337" t="s" s="0">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B338" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C338" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D338" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E338" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F338" t="s" s="0">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B339" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C339" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D339" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E339" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F339" t="s" s="0">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B340" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C340" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D340" t="s" s="0">
+        <v>523</v>
+      </c>
+      <c r="E340" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F340" t="s" s="0">
+        <v>524</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Test result report fixed database error
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="605">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -1652,6 +1652,260 @@
   </si>
   <si>
     <t>2026-10-13T22:28:38.925480</t>
+  </si>
+  <si>
+    <t>Test login failed: TypeError: Failed to fetch expected [200] but found [0]</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:20.607611900</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:21.668714100</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:22.491140100</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:23.248504400</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:25.610115600</t>
+  </si>
+  <si>
+    <t>2026-10-22T21:15:26.182843500</t>
+  </si>
+  <si>
+    <t>Product 'Campus 00' remained in cart with quantity 1 after reload.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:02:51.588847600</t>
+  </si>
+  <si>
+    <t>Quantity increased to 3 and returned to 2.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:02:55.450145900</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:02:59.245530800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:02.550669500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:04.479034300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:05.274915800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:06.398544800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:08.261896100</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:09.435585300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:09.972157800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:10.365704600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:10.889327900</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:10.971162300</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1792686793219' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:15.147914700</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1792686796620'.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:19.009604</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1792686799817' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:22.211395100</t>
+  </si>
+  <si>
+    <t>Listing status changed to sold; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:25.959599700</t>
+  </si>
+  <si>
+    <t>element click intercepted: Element &lt;a class="px-6 py-3 bg-blue-600 hover:bg-blue-700 text-white rounded-md font-medium" href="/shop" data-discover="true"&gt;...&lt;/a&gt; is not clickable at point (627, 17). Other element would receive the click: &lt;div class="flex justify-between h-16 items-center"&gt;...&lt;/div&gt;
+  (Session info: chrome=155.0.8059.86)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.12.1'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Command: [8971f78629c1731d404f73a77b97b696, clickElement {id=f.441072BC16FB9FFDFE4391B9618BBBEC.d.0B8505FA59949397B4CA178AA8C5316E.e.4}]
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 155.0.8059.86, chrome: {chromedriverVersion: 155.0.8059.84 (5869fe313571..., userDataDir: C:\Users\ASHISH~1\AppData\L...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:62284}, goog:processID: 2844, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:62284/devtoo..., se:cdpVersion: 155.0.8059.86, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Element: [[ChromeDriver: chrome on windows (8971f78629c1731d404f73a77b97b696)] -&gt; xpath: //a[normalize-space()='Shop Now']]
+Session ID: 8971f78629c1731d404f73a77b97b696</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:28.822886600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:31.009537</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:32.071395500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:33.437636300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:36.412397400</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:38.202611</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:41.359212500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:41.974760400</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:44.492072600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:47.843146300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:49.918871100</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:51.552371300</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1792686832464' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:03:54.926859400</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for alert to be present
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Windows 11', os.arch: 'amd64', os.version: '10.0', java.version: '21.0.12.1'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 155.0.8059.86, chrome: {chromedriverVersion: 155.0.8059.84 (5869fe313571..., userDataDir: C:\Users\ASHISH~1\AppData\L...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:63294}, goog:processID: 13800, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: windows, proxy: Proxy(), se:cdp: ws://localhost:63294/devtoo..., se:cdpVersion: 155.0.8059.86, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: ce466637065451fd2e9e93aecc686212</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:22.662940600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:28.217002700</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:32.712779500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:35.847258200</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:37.922343600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:38.787581500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:39.742848800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:41.490365500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:42.638207300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:43.059424500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:43.423058800</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:43.945105300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:44.080782100</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1792686946103' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:48.007519500</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1792686949325'.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:51.602742500</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1792686952393' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:54.769381700</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:05:58.879950100</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:01.561396100</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:02.980539300</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:03.877761600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:04.691820600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:07.452480</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:08.880275</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:12.006591100</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:12.639161600</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:14.949889200</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:17.933500400</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:19.772764700</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:21.440987</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1792686982551' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:06:24.994849700</t>
   </si>
 </sst>
 </file>
@@ -1696,7 +1950,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F340"/>
+  <dimension ref="A1:F406"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -8499,6 +8753,1326 @@
         <v>524</v>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B341" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C341" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D341" t="s" s="0">
+        <v>525</v>
+      </c>
+      <c r="E341" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F341" t="s" s="0">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B342" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C342" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D342" t="s" s="0">
+        <v>525</v>
+      </c>
+      <c r="E342" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F342" t="s" s="0">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B343" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C343" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D343" t="s" s="0">
+        <v>525</v>
+      </c>
+      <c r="E343" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F343" t="s" s="0">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B344" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C344" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D344" t="s" s="0">
+        <v>525</v>
+      </c>
+      <c r="E344" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F344" t="s" s="0">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B345" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C345" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D345" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E345" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F345" t="s" s="0">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B346" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C346" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D346" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E346" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F346" t="s" s="0">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B347" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C347" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D347" t="s" s="0">
+        <v>532</v>
+      </c>
+      <c r="E347" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F347" t="s" s="0">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B348" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C348" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D348" t="s" s="0">
+        <v>534</v>
+      </c>
+      <c r="E348" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F348" t="s" s="0">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B349" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C349" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D349" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E349" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F349" t="s" s="0">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B350" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C350" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D350" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E350" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F350" t="s" s="0">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B351" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C351" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D351" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E351" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F351" t="s" s="0">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B352" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C352" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D352" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E352" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F352" t="s" s="0">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B353" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C353" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D353" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E353" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F353" t="s" s="0">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B354" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C354" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D354" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E354" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F354" t="s" s="0">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B355" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C355" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D355" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E355" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F355" t="s" s="0">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B356" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C356" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D356" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E356" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F356" t="s" s="0">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B357" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C357" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D357" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E357" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F357" t="s" s="0">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B358" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C358" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D358" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E358" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F358" t="s" s="0">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B359" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C359" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D359" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E359" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F359" t="s" s="0">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B360" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C360" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D360" t="s" s="0">
+        <v>547</v>
+      </c>
+      <c r="E360" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F360" t="s" s="0">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B361" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C361" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D361" t="s" s="0">
+        <v>549</v>
+      </c>
+      <c r="E361" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F361" t="s" s="0">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B362" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C362" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D362" t="s" s="0">
+        <v>551</v>
+      </c>
+      <c r="E362" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F362" t="s" s="0">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B363" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C363" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D363" t="s" s="0">
+        <v>553</v>
+      </c>
+      <c r="E363" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F363" t="s" s="0">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B364" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C364" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D364" t="s" s="0">
+        <v>555</v>
+      </c>
+      <c r="E364" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F364" t="s" s="0">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B365" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C365" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D365" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E365" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F365" t="s" s="0">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B366" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C366" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D366" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E366" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F366" t="s" s="0">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B367" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C367" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D367" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E367" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F367" t="s" s="0">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B368" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C368" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D368" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E368" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F368" t="s" s="0">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B369" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C369" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D369" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E369" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F369" t="s" s="0">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B370" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C370" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D370" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E370" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F370" t="s" s="0">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B371" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C371" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D371" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E371" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F371" t="s" s="0">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B372" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C372" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D372" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E372" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F372" t="s" s="0">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B373" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C373" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D373" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E373" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F373" t="s" s="0">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B374" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C374" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D374" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E374" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F374" t="s" s="0">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B375" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C375" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D375" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E375" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F375" t="s" s="0">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B376" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C376" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D376" t="s" s="0">
+        <v>568</v>
+      </c>
+      <c r="E376" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F376" t="s" s="0">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B377" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C377" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D377" t="s" s="0">
+        <v>570</v>
+      </c>
+      <c r="E377" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F377" t="s" s="0">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B378" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C378" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D378" t="s" s="0">
+        <v>534</v>
+      </c>
+      <c r="E378" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F378" t="s" s="0">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B379" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C379" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D379" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E379" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F379" t="s" s="0">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B380" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C380" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D380" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E380" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F380" t="s" s="0">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B381" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C381" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D381" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E381" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F381" t="s" s="0">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B382" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C382" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D382" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E382" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F382" t="s" s="0">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B383" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C383" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D383" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E383" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F383" t="s" s="0">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B384" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C384" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D384" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E384" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F384" t="s" s="0">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B385" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C385" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D385" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E385" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F385" t="s" s="0">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B386" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C386" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D386" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E386" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F386" t="s" s="0">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B387" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C387" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D387" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E387" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F387" t="s" s="0">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B388" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C388" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D388" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E388" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F388" t="s" s="0">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B389" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C389" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D389" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E389" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F389" t="s" s="0">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B390" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C390" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D390" t="s" s="0">
+        <v>584</v>
+      </c>
+      <c r="E390" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F390" t="s" s="0">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B391" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C391" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D391" t="s" s="0">
+        <v>586</v>
+      </c>
+      <c r="E391" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F391" t="s" s="0">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B392" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C392" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D392" t="s" s="0">
+        <v>588</v>
+      </c>
+      <c r="E392" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F392" t="s" s="0">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B393" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C393" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D393" t="s" s="0">
+        <v>553</v>
+      </c>
+      <c r="E393" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F393" t="s" s="0">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B394" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C394" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D394" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E394" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F394" t="s" s="0">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B395" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C395" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D395" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E395" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F395" t="s" s="0">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B396" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C396" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D396" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E396" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F396" t="s" s="0">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B397" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C397" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D397" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E397" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F397" t="s" s="0">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B398" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C398" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D398" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E398" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F398" t="s" s="0">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B399" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C399" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D399" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E399" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F399" t="s" s="0">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B400" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C400" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D400" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E400" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F400" t="s" s="0">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B401" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C401" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D401" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E401" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F401" t="s" s="0">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B402" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C402" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D402" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E402" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F402" t="s" s="0">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B403" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C403" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D403" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E403" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F403" t="s" s="0">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B404" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C404" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D404" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E404" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F404" t="s" s="0">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B405" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C405" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D405" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E405" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F405" t="s" s="0">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B406" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C406" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D406" t="s" s="0">
+        <v>603</v>
+      </c>
+      <c r="E406" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F406" t="s" s="0">
+        <v>604</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
FIxed testng.xml file uploaded
</commit_message>
<xml_diff>
--- a/test-results/selenium_test_results.xlsx
+++ b/test-results/selenium_test_results.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2460" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3510" uniqueCount="807">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -1906,6 +1906,672 @@
   </si>
   <si>
     <t>2026-10-22T22:06:24.994849700</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:27.064085</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:27.184435</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:27.583183</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:27.664729</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:28.170679</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:28.404439</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:28.623275</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:28.713042</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:28.848410</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:29.531219</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:29.961887</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:30.438776</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:31.634719</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:32.288525</t>
+  </si>
+  <si>
+    <t>Cart quantity changed after reload. expected [2] but found [3]</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:33.138341</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:33.540931</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:33.829415</t>
+  </si>
+  <si>
+    <t>Quantity increased to 2 and returned to 1.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:36.579900</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:39.537999</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:41.963883</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:42.380852</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:42.774797</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:42.823673</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:49791}, goog:processID: 8771, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:49791/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 3391dc915be71c8fc7ca68944ee87c4d</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:44.493500</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:44.559504</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:49834}, goog:processID: 8819, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:49834/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 36eea1a9466f0f5ec75a3c2ea3d4c968</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:45.509152</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1792689946209'.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:53.250915</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:55.503634</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1792689953948' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:55.975667</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:55:59.138647</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.075520</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.183225</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.314125</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.629823</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.708418</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:16.864447</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:17.022527</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:17.077878</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:18.267328</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:18.558351</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:19.062437</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:19.308384</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:19.332937</t>
+  </si>
+  <si>
+    <t>Product 'Campus 00' remained in cart with quantity 4 after reload.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:21.003098</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:21.462257</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:21.582763</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:22.896368</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:24.555565</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:27.477238</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:29.942582</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:30.371162</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:30.737152</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:30.799482</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:32.504519</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50103}, goog:processID: 9297, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50103/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 709d4d9537b6964777afcebde2a0782f</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:33.379528</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50073}, goog:processID: 9252, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50073/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 741362de31f74aabce8daea84660ff0c</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:33.893216</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:44.428865</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:44.941895</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:56:55.484957</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:06.587460</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:38.406670</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:38.515452</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:38.626978</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:38.935252</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:39.235715</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:39.352313</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:39.381582</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:39.522176</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:39.889112</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:40.690092</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:40.926013</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:43.114502</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:44.372902</t>
+  </si>
+  <si>
+    <t>Product 'Campus 00' remained in cart with quantity 3 after reload.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:44.743081</t>
+  </si>
+  <si>
+    <t>Quantity increased to 5 and returned to 4.</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:48.268133</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:51.235021</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:53.681157</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50312}, goog:processID: 9716, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50312/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 86319eca923258de023e91b330c4a4fb</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:57:55.334614</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50380}, goog:processID: 9784, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50380/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 9e6c21219b807a83df2b69a448dd7a70</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:05.471843</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:06.402079</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:06.835018</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:06.883886</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:16.557058</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:27.632389</t>
+  </si>
+  <si>
+    <t>2026-10-22T22:58:38.725513</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:04.657715</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:04.818687</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:05.595599</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:05.866923</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:05.931513</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:06.374665</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:06.521537</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:06.708388</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:06.880461</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:07.393427</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:07.447237</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:08.291412</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:08.326215</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:10.416786</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:10.492247</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:11.678791</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for tests.CartTest$$Lambda/0x000003fe015dec00@385a5ffc
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50571}, goog:processID: 10205, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50571/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 66595470e58a4769bf9cfef8f2490ba6</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:20.682455</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50635}, goog:processID: 10295, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50635/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: a69a34ff120c22273227e5ececb9144b</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:22.122231</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:50606}, goog:processID: 10248, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:50606/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: f090d5041007be4b848d752bbad94768</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:22.716635</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:24.157954</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:27.110604</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:29.559005</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:29.991009</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:30.366710</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:30.429782</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:32.134550</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:33.090631</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:33.716509</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:44.134471</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:00:55.201668</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:11.431627</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:11.588501</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:11.697037</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.003435</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.087548</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.220899</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.347389</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.498707</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:12.706778</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:13.238328</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:13.992717</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:14.227841</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:14.997674</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:16.284705</t>
+  </si>
+  <si>
+    <t>Cart quantity changed after reload. expected [3] but found [4]</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:16.474216</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:17.165429</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:17.544990</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:18.851804</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:19.909194</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1792690399538' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:21.376030</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:21.784384</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:22.156346</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:22.217738</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:22.779850</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:23.916784</t>
+  </si>
+  <si>
+    <t>Subtotal ₹13000.00 + shipping ₹150.00 = total ₹13150.00.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:25.217182</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1792690398621' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:27.636898</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1792690408899'.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:30.737019</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1792690411447' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:33.352776</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:36.482811</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:50.005297</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:50.305720</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:50.795034</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:51.463775</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:52.193981</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:52.371226</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:52.516762</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:52.847152</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:53.169824</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:53.265619</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:53.301596</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:53.400713</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:53.528308</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:55.523329</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:55.951495</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:57.272520</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:57.291966</t>
+  </si>
+  <si>
+    <t>Cancelled deletion and listing 'Selenium QA Item 1792690437165' remained visible.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:03:58.520735</t>
+  </si>
+  <si>
+    <t>Confirmed deletion removed listing 'Selenium QA Item 1792690439779'.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:01.622148</t>
+  </si>
+  <si>
+    <t>Listing 'Selenium QA Item 1792690442324' belongs to the authenticated test user; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:04.223193</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:07.371152</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:07.795944</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:08.152120</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:08.214264</t>
+  </si>
+  <si>
+    <t>Expected condition failed: waiting for visibility of element found by By.xpath: //h2[normalize-space()='List Your Item for Sale']
+(tried for 10 seconds with 500 milliseconds interval)
+Build info: version: '4.49.0', revision: 'bedb24f bedb24f6f703876e7e4c5d506f0d697eb358c720'
+System info: os.name: 'Mac OS X', os.arch: 'aarch64', os.version: '27.0.1', java.version: '27'
+Driver info: org.openqa.selenium.chrome.ChromeDriver
+Capabilities {acceptInsecureCerts: false, browserName: chrome, browserVersion: 156.0.8078.47, chrome: {chromedriverVersion: 156.0.8078.47 (1d17a2e2ee14..., userDataDir: /var/folders/vm/0q10x59x525...}, fedcm:accounts: true, goog:chromeOptions: {debuggerAddress: localhost:51128}, goog:processID: 11237, networkConnectionEnabled: false, pageLoadStrategy: normal, platformName: mac, proxy: Proxy(), se:cdp: ws://localhost:51128/devtoo..., se:cdpVersion: 156.0.8078.47, setWindowRect: true, strictFileInteractability: false, timeouts: {implicit: 0, pageLoad: 300000, script: 30000}, unhandledPromptBehavior: dismiss and notify, webauthn:extension:cmtgKey: true, webauthn:extension:credBlob: true, webauthn:extension:largeBlob: true, webauthn:extension:minPinLength: true, webauthn:extension:prf: true, webauthn:virtualAuthenticators: true}
+Session ID: 8395ce94b5e72521cfb5020621946e57</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:08.569891</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:09.889244</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:10.429509</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:13.394828</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:15.840407</t>
+  </si>
+  <si>
+    <t>Created listing 'Selenium QA Item 1792690449270' was found in My Listings; test data cleaned up.</t>
+  </si>
+  <si>
+    <t>2026-10-22T23:04:18.334443</t>
   </si>
 </sst>
 </file>
@@ -1950,7 +2616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F406"/>
+  <dimension ref="A1:F581"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -10073,6 +10739,3506 @@
         <v>604</v>
       </c>
     </row>
+    <row r="407">
+      <c r="A407" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B407" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C407" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D407" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E407" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F407" t="s" s="0">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B408" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C408" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D408" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E408" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F408" t="s" s="0">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B409" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C409" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D409" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E409" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F409" t="s" s="0">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B410" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C410" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D410" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E410" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F410" t="s" s="0">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B411" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C411" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D411" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E411" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F411" t="s" s="0">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B412" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C412" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D412" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E412" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F412" t="s" s="0">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B413" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C413" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D413" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E413" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F413" t="s" s="0">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B414" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C414" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D414" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E414" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F414" t="s" s="0">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B415" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C415" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D415" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E415" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F415" t="s" s="0">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B416" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C416" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D416" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E416" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F416" t="s" s="0">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B417" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C417" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D417" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E417" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F417" t="s" s="0">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B418" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C418" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D418" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E418" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F418" t="s" s="0">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B419" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C419" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D419" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E419" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F419" t="s" s="0">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B420" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C420" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D420" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E420" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F420" t="s" s="0">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B421" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C421" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D421" t="s" s="0">
+        <v>619</v>
+      </c>
+      <c r="E421" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F421" t="s" s="0">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B422" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C422" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D422" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E422" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F422" t="s" s="0">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B423" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C423" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D423" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E423" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F423" t="s" s="0">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B424" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C424" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D424" t="s" s="0">
+        <v>623</v>
+      </c>
+      <c r="E424" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F424" t="s" s="0">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B425" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C425" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D425" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E425" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F425" t="s" s="0">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B426" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C426" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D426" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E426" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F426" t="s" s="0">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B427" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C427" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D427" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E427" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F427" t="s" s="0">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B428" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C428" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D428" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E428" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F428" t="s" s="0">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B429" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C429" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D429" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E429" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F429" t="s" s="0">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B430" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C430" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D430" t="s" s="0">
+        <v>630</v>
+      </c>
+      <c r="E430" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F430" t="s" s="0">
+        <v>631</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B431" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C431" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D431" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E431" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F431" t="s" s="0">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B432" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C432" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D432" t="s" s="0">
+        <v>633</v>
+      </c>
+      <c r="E432" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F432" t="s" s="0">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B433" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C433" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D433" t="s" s="0">
+        <v>635</v>
+      </c>
+      <c r="E433" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F433" t="s" s="0">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B434" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C434" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D434" t="s" s="0">
+        <v>630</v>
+      </c>
+      <c r="E434" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F434" t="s" s="0">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B435" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C435" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D435" t="s" s="0">
+        <v>638</v>
+      </c>
+      <c r="E435" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F435" t="s" s="0">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B436" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C436" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D436" t="s" s="0">
+        <v>553</v>
+      </c>
+      <c r="E436" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F436" t="s" s="0">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B437" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C437" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D437" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E437" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F437" t="s" s="0">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B438" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C438" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D438" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E438" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F438" t="s" s="0">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B439" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C439" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D439" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E439" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F439" t="s" s="0">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B440" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C440" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D440" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E440" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F440" t="s" s="0">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B441" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C441" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D441" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E441" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F441" t="s" s="0">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B442" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C442" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D442" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E442" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F442" t="s" s="0">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B443" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C443" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D443" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E443" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F443" t="s" s="0">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B444" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C444" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D444" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E444" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F444" t="s" s="0">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B445" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C445" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D445" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E445" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F445" t="s" s="0">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B446" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C446" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D446" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E446" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F446" t="s" s="0">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B447" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C447" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D447" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E447" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F447" t="s" s="0">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B448" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C448" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D448" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E448" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F448" t="s" s="0">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B449" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C449" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D449" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E449" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F449" t="s" s="0">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B450" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C450" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D450" t="s" s="0">
+        <v>654</v>
+      </c>
+      <c r="E450" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F450" t="s" s="0">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B451" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C451" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D451" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E451" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F451" t="s" s="0">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B452" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C452" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D452" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E452" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F452" t="s" s="0">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B453" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C453" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D453" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E453" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F453" t="s" s="0">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B454" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C454" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D454" t="s" s="0">
+        <v>623</v>
+      </c>
+      <c r="E454" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F454" t="s" s="0">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B455" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C455" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D455" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E455" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F455" t="s" s="0">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B456" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C456" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D456" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E456" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F456" t="s" s="0">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B457" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C457" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D457" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E457" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F457" t="s" s="0">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B458" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C458" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D458" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E458" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F458" t="s" s="0">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B459" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C459" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D459" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E459" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F459" t="s" s="0">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B460" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C460" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D460" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E460" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F460" t="s" s="0">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B461" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C461" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D461" t="s" s="0">
+        <v>666</v>
+      </c>
+      <c r="E461" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F461" t="s" s="0">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B462" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C462" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D462" t="s" s="0">
+        <v>668</v>
+      </c>
+      <c r="E462" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F462" t="s" s="0">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B463" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C463" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D463" t="s" s="0">
+        <v>666</v>
+      </c>
+      <c r="E463" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F463" t="s" s="0">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B464" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C464" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D464" t="s" s="0">
+        <v>668</v>
+      </c>
+      <c r="E464" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F464" t="s" s="0">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B465" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C465" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D465" t="s" s="0">
+        <v>666</v>
+      </c>
+      <c r="E465" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F465" t="s" s="0">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B466" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C466" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D466" t="s" s="0">
+        <v>666</v>
+      </c>
+      <c r="E466" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F466" t="s" s="0">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B467" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C467" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D467" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E467" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F467" t="s" s="0">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B468" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C468" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D468" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E468" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F468" t="s" s="0">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B469" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C469" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D469" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E469" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F469" t="s" s="0">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B470" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C470" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D470" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E470" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F470" t="s" s="0">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B471" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C471" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D471" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E471" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F471" t="s" s="0">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B472" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C472" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D472" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E472" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F472" t="s" s="0">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B473" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C473" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D473" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E473" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F473" t="s" s="0">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B474" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C474" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D474" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E474" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F474" t="s" s="0">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B475" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C475" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D475" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E475" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F475" t="s" s="0">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B476" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C476" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D476" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E476" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F476" t="s" s="0">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B477" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C477" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D477" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E477" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F477" t="s" s="0">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B478" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C478" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D478" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E478" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F478" t="s" s="0">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B479" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C479" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D479" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E479" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F479" t="s" s="0">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B480" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C480" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D480" t="s" s="0">
+        <v>687</v>
+      </c>
+      <c r="E480" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F480" t="s" s="0">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B481" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C481" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D481" t="s" s="0">
+        <v>689</v>
+      </c>
+      <c r="E481" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F481" t="s" s="0">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B482" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C482" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D482" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E482" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F482" t="s" s="0">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B483" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C483" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D483" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E483" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F483" t="s" s="0">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B484" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C484" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D484" t="s" s="0">
+        <v>693</v>
+      </c>
+      <c r="E484" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F484" t="s" s="0">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B485" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C485" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D485" t="s" s="0">
+        <v>695</v>
+      </c>
+      <c r="E485" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F485" t="s" s="0">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B486" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C486" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D486" t="s" s="0">
+        <v>693</v>
+      </c>
+      <c r="E486" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F486" t="s" s="0">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B487" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C487" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D487" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E487" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F487" t="s" s="0">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B488" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C488" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D488" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E488" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F488" t="s" s="0">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B489" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C489" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D489" t="s" s="0">
+        <v>695</v>
+      </c>
+      <c r="E489" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F489" t="s" s="0">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B490" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C490" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D490" t="s" s="0">
+        <v>695</v>
+      </c>
+      <c r="E490" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F490" t="s" s="0">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B491" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C491" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D491" t="s" s="0">
+        <v>695</v>
+      </c>
+      <c r="E491" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F491" t="s" s="0">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B492" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C492" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D492" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E492" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F492" t="s" s="0">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B493" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C493" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D493" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E493" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F493" t="s" s="0">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B494" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C494" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D494" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E494" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F494" t="s" s="0">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B495" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C495" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D495" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E495" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F495" t="s" s="0">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B496" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C496" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D496" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E496" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F496" t="s" s="0">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B497" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C497" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D497" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E497" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F497" t="s" s="0">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B498" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C498" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D498" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E498" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F498" t="s" s="0">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B499" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C499" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D499" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E499" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F499" t="s" s="0">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B500" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C500" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D500" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E500" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F500" t="s" s="0">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B501" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C501" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D501" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E501" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F501" t="s" s="0">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B502" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C502" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D502" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E502" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F502" t="s" s="0">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B503" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C503" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D503" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E503" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F503" t="s" s="0">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B504" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C504" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D504" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E504" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F504" t="s" s="0">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B505" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C505" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D505" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E505" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F505" t="s" s="0">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B506" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C506" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D506" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E506" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F506" t="s" s="0">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B507" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C507" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D507" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E507" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F507" t="s" s="0">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B508" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C508" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D508" t="s" s="0">
+        <v>719</v>
+      </c>
+      <c r="E508" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F508" t="s" s="0">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B509" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C509" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D509" t="s" s="0">
+        <v>721</v>
+      </c>
+      <c r="E509" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F509" t="s" s="0">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B510" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C510" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D510" t="s" s="0">
+        <v>723</v>
+      </c>
+      <c r="E510" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F510" t="s" s="0">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B511" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C511" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D511" t="s" s="0">
+        <v>623</v>
+      </c>
+      <c r="E511" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F511" t="s" s="0">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B512" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C512" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D512" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E512" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F512" t="s" s="0">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B513" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C513" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D513" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E513" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F513" t="s" s="0">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B514" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C514" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D514" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E514" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F514" t="s" s="0">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B515" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C515" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D515" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E515" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F515" t="s" s="0">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B516" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C516" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D516" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E516" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F516" t="s" s="0">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B517" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C517" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D517" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E517" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F517" t="s" s="0">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B518" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C518" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D518" t="s" s="0">
+        <v>721</v>
+      </c>
+      <c r="E518" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F518" t="s" s="0">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B519" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C519" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D519" t="s" s="0">
+        <v>723</v>
+      </c>
+      <c r="E519" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F519" t="s" s="0">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B520" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C520" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D520" t="s" s="0">
+        <v>721</v>
+      </c>
+      <c r="E520" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F520" t="s" s="0">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B521" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C521" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D521" t="s" s="0">
+        <v>721</v>
+      </c>
+      <c r="E521" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F521" t="s" s="0">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B522" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C522" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D522" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E522" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F522" t="s" s="0">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B523" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C523" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D523" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E523" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F523" t="s" s="0">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B524" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C524" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D524" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E524" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F524" t="s" s="0">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B525" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C525" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D525" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E525" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F525" t="s" s="0">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B526" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C526" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D526" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E526" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F526" t="s" s="0">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B527" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C527" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D527" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E527" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F527" t="s" s="0">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B528" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C528" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D528" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E528" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F528" t="s" s="0">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B529" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C529" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D529" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E529" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F529" t="s" s="0">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B530" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C530" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D530" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E530" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F530" t="s" s="0">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B531" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C531" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D531" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E531" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F531" t="s" s="0">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B532" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C532" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D532" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E532" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F532" t="s" s="0">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B533" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C533" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D533" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E533" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F533" t="s" s="0">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B534" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C534" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D534" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E534" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F534" t="s" s="0">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B535" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C535" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D535" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E535" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F535" t="s" s="0">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B536" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C536" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D536" t="s" s="0">
+        <v>750</v>
+      </c>
+      <c r="E536" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F536" t="s" s="0">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B537" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C537" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D537" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E537" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F537" t="s" s="0">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B538" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C538" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D538" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E538" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F538" t="s" s="0">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B539" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C539" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D539" t="s" s="0">
+        <v>280</v>
+      </c>
+      <c r="E539" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F539" t="s" s="0">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B540" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C540" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D540" t="s" s="0">
+        <v>623</v>
+      </c>
+      <c r="E540" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F540" t="s" s="0">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B541" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C541" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D541" t="s" s="0">
+        <v>756</v>
+      </c>
+      <c r="E541" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F541" t="s" s="0">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B542" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C542" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D542" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E542" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F542" t="s" s="0">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B543" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C543" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D543" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E543" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F543" t="s" s="0">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B544" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C544" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D544" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E544" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F544" t="s" s="0">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B545" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C545" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D545" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E545" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F545" t="s" s="0">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B546" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C546" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D546" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E546" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F546" t="s" s="0">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B547" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C547" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D547" t="s" s="0">
+        <v>763</v>
+      </c>
+      <c r="E547" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F547" t="s" s="0">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B548" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C548" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D548" t="s" s="0">
+        <v>765</v>
+      </c>
+      <c r="E548" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F548" t="s" s="0">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B549" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C549" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D549" t="s" s="0">
+        <v>767</v>
+      </c>
+      <c r="E549" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F549" t="s" s="0">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B550" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C550" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D550" t="s" s="0">
+        <v>769</v>
+      </c>
+      <c r="E550" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F550" t="s" s="0">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B551" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C551" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D551" t="s" s="0">
+        <v>553</v>
+      </c>
+      <c r="E551" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F551" t="s" s="0">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B552" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C552" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D552" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E552" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F552" t="s" s="0">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="s" s="0">
+        <v>244</v>
+      </c>
+      <c r="B553" t="s" s="0">
+        <v>245</v>
+      </c>
+      <c r="C553" t="s" s="0">
+        <v>246</v>
+      </c>
+      <c r="D553" t="s" s="0">
+        <v>247</v>
+      </c>
+      <c r="E553" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F553" t="s" s="0">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="s" s="0">
+        <v>249</v>
+      </c>
+      <c r="B554" t="s" s="0">
+        <v>250</v>
+      </c>
+      <c r="C554" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="D554" t="s" s="0">
+        <v>252</v>
+      </c>
+      <c r="E554" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F554" t="s" s="0">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="B555" t="s" s="0">
+        <v>437</v>
+      </c>
+      <c r="C555" t="s" s="0">
+        <v>438</v>
+      </c>
+      <c r="D555" t="s" s="0">
+        <v>439</v>
+      </c>
+      <c r="E555" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F555" t="s" s="0">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B556" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C556" t="s" s="0">
+        <v>441</v>
+      </c>
+      <c r="D556" t="s" s="0">
+        <v>442</v>
+      </c>
+      <c r="E556" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F556" t="s" s="0">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="B557" t="s" s="0">
+        <v>173</v>
+      </c>
+      <c r="C557" t="s" s="0">
+        <v>174</v>
+      </c>
+      <c r="D557" t="s" s="0">
+        <v>175</v>
+      </c>
+      <c r="E557" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F557" t="s" s="0">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B558" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C558" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D558" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="E558" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F558" t="s" s="0">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="B559" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="C559" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="D559" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="E559" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F559" t="s" s="0">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B560" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C560" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D560" t="s" s="0">
+        <v>83</v>
+      </c>
+      <c r="E560" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F560" t="s" s="0">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B561" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C561" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="D561" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E561" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F561" t="s" s="0">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B562" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C562" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="D562" t="s" s="0">
+        <v>81</v>
+      </c>
+      <c r="E562" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F562" t="s" s="0">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="s" s="0">
+        <v>206</v>
+      </c>
+      <c r="B563" t="s" s="0">
+        <v>207</v>
+      </c>
+      <c r="C563" t="s" s="0">
+        <v>208</v>
+      </c>
+      <c r="D563" t="s" s="0">
+        <v>209</v>
+      </c>
+      <c r="E563" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F563" t="s" s="0">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="s" s="0">
+        <v>261</v>
+      </c>
+      <c r="B564" t="s" s="0">
+        <v>262</v>
+      </c>
+      <c r="C564" t="s" s="0">
+        <v>263</v>
+      </c>
+      <c r="D564" t="s" s="0">
+        <v>264</v>
+      </c>
+      <c r="E564" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F564" t="s" s="0">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="s" s="0">
+        <v>157</v>
+      </c>
+      <c r="B565" t="s" s="0">
+        <v>158</v>
+      </c>
+      <c r="C565" t="s" s="0">
+        <v>159</v>
+      </c>
+      <c r="D565" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="E565" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F565" t="s" s="0">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="s" s="0">
+        <v>329</v>
+      </c>
+      <c r="B566" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="C566" t="s" s="0">
+        <v>331</v>
+      </c>
+      <c r="D566" t="s" s="0">
+        <v>332</v>
+      </c>
+      <c r="E566" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F566" t="s" s="0">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B567" t="s" s="0">
+        <v>219</v>
+      </c>
+      <c r="C567" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="D567" t="s" s="0">
+        <v>532</v>
+      </c>
+      <c r="E567" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F567" t="s" s="0">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="s" s="0">
+        <v>334</v>
+      </c>
+      <c r="B568" t="s" s="0">
+        <v>335</v>
+      </c>
+      <c r="C568" t="s" s="0">
+        <v>336</v>
+      </c>
+      <c r="D568" t="s" s="0">
+        <v>337</v>
+      </c>
+      <c r="E568" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F568" t="s" s="0">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="s" s="0">
+        <v>301</v>
+      </c>
+      <c r="B569" t="s" s="0">
+        <v>302</v>
+      </c>
+      <c r="C569" t="s" s="0">
+        <v>303</v>
+      </c>
+      <c r="D569" t="s" s="0">
+        <v>789</v>
+      </c>
+      <c r="E569" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F569" t="s" s="0">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="s" s="0">
+        <v>306</v>
+      </c>
+      <c r="B570" t="s" s="0">
+        <v>307</v>
+      </c>
+      <c r="C570" t="s" s="0">
+        <v>308</v>
+      </c>
+      <c r="D570" t="s" s="0">
+        <v>791</v>
+      </c>
+      <c r="E570" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F570" t="s" s="0">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="B571" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="C571" t="s" s="0">
+        <v>313</v>
+      </c>
+      <c r="D571" t="s" s="0">
+        <v>793</v>
+      </c>
+      <c r="E571" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F571" t="s" s="0">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="s" s="0">
+        <v>316</v>
+      </c>
+      <c r="B572" t="s" s="0">
+        <v>317</v>
+      </c>
+      <c r="C572" t="s" s="0">
+        <v>318</v>
+      </c>
+      <c r="D572" t="s" s="0">
+        <v>553</v>
+      </c>
+      <c r="E572" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F572" t="s" s="0">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B573" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C573" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="D573" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E573" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F573" t="s" s="0">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="s" s="0">
+        <v>85</v>
+      </c>
+      <c r="B574" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="C574" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="D574" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="E574" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F574" t="s" s="0">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B575" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C575" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="D575" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E575" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F575" t="s" s="0">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="s" s="0">
+        <v>277</v>
+      </c>
+      <c r="B576" t="s" s="0">
+        <v>278</v>
+      </c>
+      <c r="C576" t="s" s="0">
+        <v>279</v>
+      </c>
+      <c r="D576" t="s" s="0">
+        <v>799</v>
+      </c>
+      <c r="E576" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F576" t="s" s="0">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="s" s="0">
+        <v>90</v>
+      </c>
+      <c r="B577" t="s" s="0">
+        <v>91</v>
+      </c>
+      <c r="C577" t="s" s="0">
+        <v>92</v>
+      </c>
+      <c r="D577" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E577" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F577" t="s" s="0">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="s" s="0">
+        <v>223</v>
+      </c>
+      <c r="B578" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="C578" t="s" s="0">
+        <v>225</v>
+      </c>
+      <c r="D578" t="s" s="0">
+        <v>534</v>
+      </c>
+      <c r="E578" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F578" t="s" s="0">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="s" s="0">
+        <v>227</v>
+      </c>
+      <c r="B579" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="C579" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="D579" t="s" s="0">
+        <v>239</v>
+      </c>
+      <c r="E579" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F579" t="s" s="0">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="s" s="0">
+        <v>231</v>
+      </c>
+      <c r="B580" t="s" s="0">
+        <v>232</v>
+      </c>
+      <c r="C580" t="s" s="0">
+        <v>233</v>
+      </c>
+      <c r="D580" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="E580" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F580" t="s" s="0">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="s" s="0">
+        <v>282</v>
+      </c>
+      <c r="B581" t="s" s="0">
+        <v>283</v>
+      </c>
+      <c r="C581" t="s" s="0">
+        <v>284</v>
+      </c>
+      <c r="D581" t="s" s="0">
+        <v>805</v>
+      </c>
+      <c r="E581" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="F581" t="s" s="0">
+        <v>806</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>